<commit_message>
feat: balance combat consequences and release v0.8.2
</commit_message>
<xml_diff>
--- a/docs/data/balance-rules.xlsx
+++ b/docs/data/balance-rules.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R037e527f8efe4354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BalanceRules" sheetId="2" r:id="R9324cf74bdf64481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R324ce0afd968496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BalanceRules" sheetId="2" r:id="R89156b32e673479f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1183,6 +1183,91 @@
         <x:v>资源主键已切换为 UUID；v2、v3、v4 存档全部作废且不迁移</x:v>
       </x:c>
     </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>技能</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>绝招成长硬锁</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>仅接受当前门派、装备与等级解锁列表中的标准绝招 ID</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>门派架构30级解锁一档，80级解锁二档；执行前按ID重新解析权威配置</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>外部字典不能伪造能力、精力消耗或等级绕过门槛</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>技能</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>绝招两档平衡</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>一档效果等级最多74；二档使用完整功力</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>effect_level = min(innerLevel,74)（一档）/ innerLevel（二档）</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>80级后形成低耗稳定与高耗完整的选择，不再是同效果不同价格</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>AI</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>角色化意图决策</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>striker偏加力；controller偏绝招；tank偏恢复；其余原型各有概率曲线</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>combatRole默认行为可由ai.ultUseRate/forceUseRate/restUseRate/itemUseRate覆盖</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>下一回合意图先写入【预判】战报；原型不直接修改攻防命中或伤害</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>人物</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>NPC击败后果</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>静态NPC冷却300游戏秒，累计落败次数随v5角色存档保持</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>defeated_until + defeat_counts；动态任务NPC仍只保留本局状态</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>胜利立即安全保存；复出后对白与人物详情反馈历史交手</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>发布</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>发布前闸门</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>数据/预设/文件规模/Godot全量测试全部通过</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>npm run release:check</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>测试先完整--import，使用/tmp日志与存档，逐例90秒超时并扫描脚本加载错误</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>